<commit_message>
chore: sync Nova upm-release-2026.07.29-01
</commit_message>
<xml_diff>
--- a/Assets/Samples/AIHelpDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
+++ b/Assets/Samples/AIHelpDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
@@ -1181,7 +1181,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
   <dimension ref="A1:U44"/>
   <sheetFormatPr defaultColWidth="13" defaultRowHeight="16.8"/>
@@ -1471,7 +1471,33 @@
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
     </row>
-    <row r="10" ht="22" customHeight="1"/>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>AppCustomConfig</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>拉取GM后台应用配置URL</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>HTTP_POST</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>GameServer</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>/v1/common/app-config</t>
+        </is>
+      </c>
+    </row>
     <row r="11" ht="22" customHeight="1"/>
     <row r="12" ht="22" customHeight="1"/>
     <row r="13" ht="22" customHeight="1"/>

</xml_diff>